<commit_message>
sql qns done 30 and bit manipulation done
</commit_message>
<xml_diff>
--- a/blind 75.xlsx
+++ b/blind 75.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dhruv\OneDrive\Desktop\strivers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32B82279-55A4-4D50-A13D-0A0322DD35F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62B4AAAE-3050-42EB-BDF3-F7FEF791EF42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -717,27 +717,27 @@
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A15" s="2" t="s">
+      <c r="A15" s="4" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A16" s="2" t="s">
+      <c r="A16" s="4" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A17" s="2" t="s">
+      <c r="A17" s="4" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A18" s="2" t="s">
+      <c r="A18" s="4" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A19" s="2" t="s">
+      <c r="A19" s="4" t="s">
         <v>16</v>
       </c>
     </row>
@@ -758,7 +758,7 @@
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A24" s="2" t="s">
+      <c r="A24" s="4" t="s">
         <v>19</v>
       </c>
     </row>
@@ -773,12 +773,12 @@
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A27" s="2" t="s">
+      <c r="A27" s="4" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A28" s="2" t="s">
+      <c r="A28" s="4" t="s">
         <v>23</v>
       </c>
     </row>
@@ -793,7 +793,7 @@
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A31" s="2" t="s">
+      <c r="A31" s="4" t="s">
         <v>26</v>
       </c>
     </row>
@@ -803,7 +803,7 @@
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A33" s="2" t="s">
+      <c r="A33" s="4" t="s">
         <v>28</v>
       </c>
     </row>

</xml_diff>